<commit_message>
chore(rdm): update Interface_RDM, Scenario1, Model_Structure and ignore /Results
- Interface_RDM.xlsx: actualizaciones de configuracion del modelo
- Scenario1.txt: actualizacion de sets/parametros del escenario base
- B1_Model_Structure.xlsx: ajustes en estructura del experimento
- .gitignore: ignorar carpeta /Results
</commit_message>
<xml_diff>
--- a/src/workflow/1_Experiment/0_From_Confection/B1_Model_Structure.xlsx
+++ b/src/workflow/1_Experiment/0_From_Confection/B1_Model_Structure.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="779">
   <si>
     <t>set</t>
   </si>
@@ -111,6 +111,15 @@
     <t>u</t>
   </si>
   <si>
+    <t>DUMMYLUCF</t>
+  </si>
+  <si>
+    <t>DAC</t>
+  </si>
+  <si>
+    <t>INDPLANTOTHCCS</t>
+  </si>
+  <si>
     <t>DUMREWET</t>
   </si>
   <si>
@@ -1206,6 +1215,15 @@
     <t>S24</t>
   </si>
   <si>
+    <t>DUMLUCF</t>
+  </si>
+  <si>
+    <t>DACCO2</t>
+  </si>
+  <si>
+    <t>EXPELC</t>
+  </si>
+  <si>
     <t>PWRWAT0</t>
   </si>
   <si>
@@ -1677,6 +1695,9 @@
     <t>EXTWST</t>
   </si>
   <si>
+    <t>EXTECO</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -1812,9 +1833,6 @@
     <t>DEFORBAL</t>
   </si>
   <si>
-    <t>LNDGRSBAL</t>
-  </si>
-  <si>
     <t>2TRACAREVCAP</t>
   </si>
   <si>
@@ -1839,9 +1857,6 @@
     <t>RECWST</t>
   </si>
   <si>
-    <t>RESTRICTWAT</t>
-  </si>
-  <si>
     <t>TRADSLHTRCURCAP</t>
   </si>
   <si>
@@ -1870,6 +1885,24 @@
   </si>
   <si>
     <t>INDOTHLPHELCSHARE</t>
+  </si>
+  <si>
+    <t>PWRCOA003BAL</t>
+  </si>
+  <si>
+    <t>INDMINHPHCAP</t>
+  </si>
+  <si>
+    <t>INDCEMKILNCAP</t>
+  </si>
+  <si>
+    <t>INDASHPLANTCAP</t>
+  </si>
+  <si>
+    <t>INDASHHPHCAP</t>
+  </si>
+  <si>
+    <t>INDOTHPLANTCAP</t>
   </si>
   <si>
     <t>category</t>
@@ -2651,7 +2684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O360"/>
+  <dimension ref="A1:O363"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -2756,16 +2789,16 @@
         <v>36</v>
       </c>
       <c r="C3">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D3">
         <v>8</v>
       </c>
       <c r="E3">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -2792,7 +2825,7 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -2803,37 +2836,37 @@
         <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="E4" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="F4" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="G4" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="H4" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="I4" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="J4" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="K4" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="L4" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="M4" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="O4" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -2844,22 +2877,22 @@
         <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E5" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="F5" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="I5" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="K5" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="O5" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -2870,19 +2903,19 @@
         <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="E6" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="F6" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="K6" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="O6" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -2893,19 +2926,19 @@
         <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="E7" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="F7" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="K7" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="O7" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -2916,19 +2949,19 @@
         <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="E8" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="F8" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="K8" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="O8" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -2939,19 +2972,19 @@
         <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="E9" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="F9" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="K9" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="O9" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -2962,19 +2995,19 @@
         <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="E10" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="F10" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="K10" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="O10" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -2985,19 +3018,19 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="E11" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F11" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="K11" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="O11" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -3008,13 +3041,13 @@
         <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="F12" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="O12" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -3025,13 +3058,13 @@
         <v>40</v>
       </c>
       <c r="E13" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="F13" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="O13" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -3042,13 +3075,13 @@
         <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="F14" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="O14" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -3059,13 +3092,13 @@
         <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F15" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="O15" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -3076,10 +3109,13 @@
         <v>43</v>
       </c>
       <c r="E16" t="s">
-        <v>408</v>
+        <v>411</v>
+      </c>
+      <c r="F16" t="s">
+        <v>559</v>
       </c>
       <c r="O16" t="s">
-        <v>575</v>
+        <v>582</v>
       </c>
     </row>
     <row r="17" spans="2:15">
@@ -3090,10 +3126,10 @@
         <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="O17" t="s">
-        <v>576</v>
+        <v>583</v>
       </c>
     </row>
     <row r="18" spans="2:15">
@@ -3104,10 +3140,10 @@
         <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="O18" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
     </row>
     <row r="19" spans="2:15">
@@ -3118,10 +3154,10 @@
         <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="O19" t="s">
-        <v>578</v>
+        <v>585</v>
       </c>
     </row>
     <row r="20" spans="2:15">
@@ -3132,10 +3168,10 @@
         <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="O20" t="s">
-        <v>579</v>
+        <v>586</v>
       </c>
     </row>
     <row r="21" spans="2:15">
@@ -3146,10 +3182,10 @@
         <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="O21" t="s">
-        <v>580</v>
+        <v>587</v>
       </c>
     </row>
     <row r="22" spans="2:15">
@@ -3160,10 +3196,10 @@
         <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="O22" t="s">
-        <v>581</v>
+        <v>588</v>
       </c>
     </row>
     <row r="23" spans="2:15">
@@ -3174,10 +3210,10 @@
         <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="O23" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
     </row>
     <row r="24" spans="2:15">
@@ -3188,10 +3224,10 @@
         <v>51</v>
       </c>
       <c r="E24" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="O24" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
     </row>
     <row r="25" spans="2:15">
@@ -3202,10 +3238,10 @@
         <v>52</v>
       </c>
       <c r="E25" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="O25" t="s">
-        <v>584</v>
+        <v>591</v>
       </c>
     </row>
     <row r="26" spans="2:15">
@@ -3216,10 +3252,10 @@
         <v>53</v>
       </c>
       <c r="E26" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="O26" t="s">
-        <v>585</v>
+        <v>592</v>
       </c>
     </row>
     <row r="27" spans="2:15">
@@ -3230,10 +3266,10 @@
         <v>54</v>
       </c>
       <c r="E27" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="O27" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
     </row>
     <row r="28" spans="2:15">
@@ -3244,10 +3280,10 @@
         <v>55</v>
       </c>
       <c r="E28" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="O28" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
     </row>
     <row r="29" spans="2:15">
@@ -3258,10 +3294,10 @@
         <v>56</v>
       </c>
       <c r="E29" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="O29" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
     </row>
     <row r="30" spans="2:15">
@@ -3272,10 +3308,10 @@
         <v>57</v>
       </c>
       <c r="E30" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="O30" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
     </row>
     <row r="31" spans="2:15">
@@ -3286,10 +3322,10 @@
         <v>58</v>
       </c>
       <c r="E31" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="O31" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
     </row>
     <row r="32" spans="2:15">
@@ -3300,10 +3336,10 @@
         <v>59</v>
       </c>
       <c r="E32" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="O32" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
     </row>
     <row r="33" spans="2:15">
@@ -3314,10 +3350,10 @@
         <v>60</v>
       </c>
       <c r="E33" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="O33" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
     </row>
     <row r="34" spans="2:15">
@@ -3328,10 +3364,10 @@
         <v>61</v>
       </c>
       <c r="E34" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="O34" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
     </row>
     <row r="35" spans="2:15">
@@ -3342,10 +3378,10 @@
         <v>62</v>
       </c>
       <c r="E35" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="O35" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
     </row>
     <row r="36" spans="2:15">
@@ -3356,10 +3392,10 @@
         <v>63</v>
       </c>
       <c r="E36" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="O36" t="s">
-        <v>595</v>
+        <v>602</v>
       </c>
     </row>
     <row r="37" spans="2:15">
@@ -3370,10 +3406,10 @@
         <v>64</v>
       </c>
       <c r="E37" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="O37" t="s">
-        <v>596</v>
+        <v>603</v>
       </c>
     </row>
     <row r="38" spans="2:15">
@@ -3384,10 +3420,10 @@
         <v>65</v>
       </c>
       <c r="E38" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="O38" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
     </row>
     <row r="39" spans="2:15">
@@ -3398,10 +3434,10 @@
         <v>66</v>
       </c>
       <c r="E39" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="O39" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
     </row>
     <row r="40" spans="2:15">
@@ -3409,10 +3445,10 @@
         <v>67</v>
       </c>
       <c r="E40" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="O40" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
     </row>
     <row r="41" spans="2:15">
@@ -3420,10 +3456,10 @@
         <v>68</v>
       </c>
       <c r="E41" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="O41" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
     </row>
     <row r="42" spans="2:15">
@@ -3431,10 +3467,10 @@
         <v>69</v>
       </c>
       <c r="E42" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="O42" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
     </row>
     <row r="43" spans="2:15">
@@ -3442,10 +3478,10 @@
         <v>70</v>
       </c>
       <c r="E43" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="O43" t="s">
-        <v>602</v>
+        <v>609</v>
       </c>
     </row>
     <row r="44" spans="2:15">
@@ -3453,10 +3489,10 @@
         <v>71</v>
       </c>
       <c r="E44" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="O44" t="s">
-        <v>603</v>
+        <v>610</v>
       </c>
     </row>
     <row r="45" spans="2:15">
@@ -3464,10 +3500,10 @@
         <v>72</v>
       </c>
       <c r="E45" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="O45" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
     </row>
     <row r="46" spans="2:15">
@@ -3475,10 +3511,10 @@
         <v>73</v>
       </c>
       <c r="E46" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="O46" t="s">
-        <v>605</v>
+        <v>612</v>
       </c>
     </row>
     <row r="47" spans="2:15">
@@ -3486,10 +3522,10 @@
         <v>74</v>
       </c>
       <c r="E47" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="O47" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="48" spans="2:15">
@@ -3497,10 +3533,10 @@
         <v>75</v>
       </c>
       <c r="E48" t="s">
-        <v>171</v>
+        <v>443</v>
       </c>
       <c r="O48" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
     </row>
     <row r="49" spans="3:15">
@@ -3508,10 +3544,10 @@
         <v>76</v>
       </c>
       <c r="E49" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="O49" t="s">
-        <v>608</v>
+        <v>615</v>
       </c>
     </row>
     <row r="50" spans="3:15">
@@ -3519,10 +3555,10 @@
         <v>77</v>
       </c>
       <c r="E50" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="O50" t="s">
-        <v>609</v>
+        <v>616</v>
       </c>
     </row>
     <row r="51" spans="3:15">
@@ -3530,10 +3566,10 @@
         <v>78</v>
       </c>
       <c r="E51" t="s">
-        <v>442</v>
+        <v>174</v>
       </c>
       <c r="O51" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
     </row>
     <row r="52" spans="3:15">
@@ -3541,10 +3577,10 @@
         <v>79</v>
       </c>
       <c r="E52" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="O52" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
     </row>
     <row r="53" spans="3:15">
@@ -3552,10 +3588,10 @@
         <v>80</v>
       </c>
       <c r="E53" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="O53" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
     </row>
     <row r="54" spans="3:15">
@@ -3563,10 +3599,10 @@
         <v>81</v>
       </c>
       <c r="E54" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="O54" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
     </row>
     <row r="55" spans="3:15">
@@ -3574,10 +3610,10 @@
         <v>82</v>
       </c>
       <c r="E55" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="O55" t="s">
-        <v>614</v>
+        <v>621</v>
       </c>
     </row>
     <row r="56" spans="3:15">
@@ -3585,10 +3621,10 @@
         <v>83</v>
       </c>
       <c r="E56" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="O56" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
     </row>
     <row r="57" spans="3:15">
@@ -3596,10 +3632,10 @@
         <v>84</v>
       </c>
       <c r="E57" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="O57" t="s">
-        <v>616</v>
+        <v>623</v>
       </c>
     </row>
     <row r="58" spans="3:15">
@@ -3607,10 +3643,10 @@
         <v>85</v>
       </c>
       <c r="E58" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="O58" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
     </row>
     <row r="59" spans="3:15">
@@ -3618,7 +3654,10 @@
         <v>86</v>
       </c>
       <c r="E59" t="s">
-        <v>450</v>
+        <v>453</v>
+      </c>
+      <c r="O59" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="60" spans="3:15">
@@ -3626,7 +3665,10 @@
         <v>87</v>
       </c>
       <c r="E60" t="s">
-        <v>451</v>
+        <v>454</v>
+      </c>
+      <c r="O60" t="s">
+        <v>626</v>
       </c>
     </row>
     <row r="61" spans="3:15">
@@ -3634,7 +3676,10 @@
         <v>88</v>
       </c>
       <c r="E61" t="s">
-        <v>452</v>
+        <v>455</v>
+      </c>
+      <c r="O61" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="62" spans="3:15">
@@ -3642,7 +3687,10 @@
         <v>89</v>
       </c>
       <c r="E62" t="s">
-        <v>453</v>
+        <v>456</v>
+      </c>
+      <c r="O62" t="s">
+        <v>628</v>
       </c>
     </row>
     <row r="63" spans="3:15">
@@ -3650,7 +3698,10 @@
         <v>90</v>
       </c>
       <c r="E63" t="s">
-        <v>454</v>
+        <v>457</v>
+      </c>
+      <c r="O63" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="64" spans="3:15">
@@ -3658,135 +3709,144 @@
         <v>91</v>
       </c>
       <c r="E64" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="65" spans="3:5">
+        <v>458</v>
+      </c>
+      <c r="O64" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="65" spans="3:15">
       <c r="C65" t="s">
         <v>92</v>
       </c>
       <c r="E65" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="66" spans="3:5">
+        <v>459</v>
+      </c>
+      <c r="O65" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="66" spans="3:15">
       <c r="C66" t="s">
         <v>93</v>
       </c>
       <c r="E66" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="67" spans="3:5">
+        <v>460</v>
+      </c>
+      <c r="O66" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="67" spans="3:15">
       <c r="C67" t="s">
         <v>94</v>
       </c>
       <c r="E67" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="68" spans="3:5">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="68" spans="3:15">
       <c r="C68" t="s">
         <v>95</v>
       </c>
       <c r="E68" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="69" spans="3:5">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="69" spans="3:15">
       <c r="C69" t="s">
         <v>96</v>
       </c>
       <c r="E69" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="70" spans="3:5">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="70" spans="3:15">
       <c r="C70" t="s">
         <v>97</v>
       </c>
       <c r="E70" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="71" spans="3:5">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="71" spans="3:15">
       <c r="C71" t="s">
         <v>98</v>
       </c>
       <c r="E71" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="72" spans="3:5">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="72" spans="3:15">
       <c r="C72" t="s">
         <v>99</v>
       </c>
       <c r="E72" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="73" spans="3:5">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="73" spans="3:15">
       <c r="C73" t="s">
         <v>100</v>
       </c>
       <c r="E73" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="74" spans="3:5">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="74" spans="3:15">
       <c r="C74" t="s">
         <v>101</v>
       </c>
       <c r="E74" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="75" spans="3:5">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="75" spans="3:15">
       <c r="C75" t="s">
         <v>102</v>
       </c>
       <c r="E75" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="76" spans="3:5">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="76" spans="3:15">
       <c r="C76" t="s">
         <v>103</v>
       </c>
       <c r="E76" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="77" spans="3:5">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="77" spans="3:15">
       <c r="C77" t="s">
         <v>104</v>
       </c>
       <c r="E77" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="78" spans="3:5">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="78" spans="3:15">
       <c r="C78" t="s">
         <v>105</v>
       </c>
       <c r="E78" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="79" spans="3:5">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="79" spans="3:15">
       <c r="C79" t="s">
         <v>106</v>
       </c>
       <c r="E79" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="80" spans="3:5">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="80" spans="3:15">
       <c r="C80" t="s">
         <v>107</v>
       </c>
       <c r="E80" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="81" spans="3:5">
@@ -3794,7 +3854,7 @@
         <v>108</v>
       </c>
       <c r="E81" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="82" spans="3:5">
@@ -3802,7 +3862,7 @@
         <v>109</v>
       </c>
       <c r="E82" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
     </row>
     <row r="83" spans="3:5">
@@ -3810,7 +3870,7 @@
         <v>110</v>
       </c>
       <c r="E83" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="84" spans="3:5">
@@ -3818,7 +3878,7 @@
         <v>111</v>
       </c>
       <c r="E84" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="85" spans="3:5">
@@ -3826,7 +3886,7 @@
         <v>112</v>
       </c>
       <c r="E85" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="86" spans="3:5">
@@ -3834,7 +3894,7 @@
         <v>113</v>
       </c>
       <c r="E86" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
     </row>
     <row r="87" spans="3:5">
@@ -3842,7 +3902,7 @@
         <v>114</v>
       </c>
       <c r="E87" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="88" spans="3:5">
@@ -3850,7 +3910,7 @@
         <v>115</v>
       </c>
       <c r="E88" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
     </row>
     <row r="89" spans="3:5">
@@ -3858,7 +3918,7 @@
         <v>116</v>
       </c>
       <c r="E89" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="90" spans="3:5">
@@ -3866,7 +3926,7 @@
         <v>117</v>
       </c>
       <c r="E90" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="91" spans="3:5">
@@ -3874,7 +3934,7 @@
         <v>118</v>
       </c>
       <c r="E91" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
     </row>
     <row r="92" spans="3:5">
@@ -3882,7 +3942,7 @@
         <v>119</v>
       </c>
       <c r="E92" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
     </row>
     <row r="93" spans="3:5">
@@ -3890,7 +3950,7 @@
         <v>120</v>
       </c>
       <c r="E93" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="94" spans="3:5">
@@ -3898,7 +3958,7 @@
         <v>121</v>
       </c>
       <c r="E94" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="95" spans="3:5">
@@ -3906,7 +3966,7 @@
         <v>122</v>
       </c>
       <c r="E95" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="96" spans="3:5">
@@ -3914,7 +3974,7 @@
         <v>123</v>
       </c>
       <c r="E96" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
     <row r="97" spans="3:5">
@@ -3922,7 +3982,7 @@
         <v>124</v>
       </c>
       <c r="E97" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="98" spans="3:5">
@@ -3930,7 +3990,7 @@
         <v>125</v>
       </c>
       <c r="E98" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="99" spans="3:5">
@@ -3938,7 +3998,7 @@
         <v>126</v>
       </c>
       <c r="E99" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="100" spans="3:5">
@@ -3946,7 +4006,7 @@
         <v>127</v>
       </c>
       <c r="E100" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="101" spans="3:5">
@@ -3954,7 +4014,7 @@
         <v>128</v>
       </c>
       <c r="E101" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="102" spans="3:5">
@@ -3962,7 +4022,7 @@
         <v>129</v>
       </c>
       <c r="E102" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
     </row>
     <row r="103" spans="3:5">
@@ -3970,7 +4030,7 @@
         <v>130</v>
       </c>
       <c r="E103" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="104" spans="3:5">
@@ -3978,7 +4038,7 @@
         <v>131</v>
       </c>
       <c r="E104" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
     </row>
     <row r="105" spans="3:5">
@@ -3986,7 +4046,7 @@
         <v>132</v>
       </c>
       <c r="E105" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="106" spans="3:5">
@@ -3994,7 +4054,7 @@
         <v>133</v>
       </c>
       <c r="E106" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="107" spans="3:5">
@@ -4002,7 +4062,7 @@
         <v>134</v>
       </c>
       <c r="E107" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="108" spans="3:5">
@@ -4010,7 +4070,7 @@
         <v>135</v>
       </c>
       <c r="E108" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
     </row>
     <row r="109" spans="3:5">
@@ -4018,7 +4078,7 @@
         <v>136</v>
       </c>
       <c r="E109" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="110" spans="3:5">
@@ -4026,7 +4086,7 @@
         <v>137</v>
       </c>
       <c r="E110" t="s">
-        <v>242</v>
+        <v>504</v>
       </c>
     </row>
     <row r="111" spans="3:5">
@@ -4034,7 +4094,7 @@
         <v>138</v>
       </c>
       <c r="E111" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
     </row>
     <row r="112" spans="3:5">
@@ -4042,7 +4102,7 @@
         <v>139</v>
       </c>
       <c r="E112" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
     </row>
     <row r="113" spans="3:5">
@@ -4050,7 +4110,7 @@
         <v>140</v>
       </c>
       <c r="E113" t="s">
-        <v>503</v>
+        <v>245</v>
       </c>
     </row>
     <row r="114" spans="3:5">
@@ -4058,7 +4118,7 @@
         <v>141</v>
       </c>
       <c r="E114" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
     </row>
     <row r="115" spans="3:5">
@@ -4066,7 +4126,7 @@
         <v>142</v>
       </c>
       <c r="E115" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
     </row>
     <row r="116" spans="3:5">
@@ -4074,7 +4134,7 @@
         <v>143</v>
       </c>
       <c r="E116" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
     </row>
     <row r="117" spans="3:5">
@@ -4082,7 +4142,7 @@
         <v>144</v>
       </c>
       <c r="E117" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="118" spans="3:5">
@@ -4090,7 +4150,7 @@
         <v>145</v>
       </c>
       <c r="E118" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
     </row>
     <row r="119" spans="3:5">
@@ -4098,7 +4158,7 @@
         <v>146</v>
       </c>
       <c r="E119" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
     </row>
     <row r="120" spans="3:5">
@@ -4106,7 +4166,7 @@
         <v>147</v>
       </c>
       <c r="E120" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row r="121" spans="3:5">
@@ -4114,7 +4174,7 @@
         <v>148</v>
       </c>
       <c r="E121" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="122" spans="3:5">
@@ -4122,7 +4182,7 @@
         <v>149</v>
       </c>
       <c r="E122" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="123" spans="3:5">
@@ -4130,7 +4190,7 @@
         <v>150</v>
       </c>
       <c r="E123" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
     </row>
     <row r="124" spans="3:5">
@@ -4138,7 +4198,7 @@
         <v>151</v>
       </c>
       <c r="E124" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
     </row>
     <row r="125" spans="3:5">
@@ -4146,7 +4206,7 @@
         <v>152</v>
       </c>
       <c r="E125" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="126" spans="3:5">
@@ -4154,7 +4214,7 @@
         <v>153</v>
       </c>
       <c r="E126" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
     </row>
     <row r="127" spans="3:5">
@@ -4162,7 +4222,7 @@
         <v>154</v>
       </c>
       <c r="E127" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
     </row>
     <row r="128" spans="3:5">
@@ -4170,7 +4230,7 @@
         <v>155</v>
       </c>
       <c r="E128" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
     </row>
     <row r="129" spans="3:5">
@@ -4178,7 +4238,7 @@
         <v>156</v>
       </c>
       <c r="E129" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
     </row>
     <row r="130" spans="3:5">
@@ -4186,7 +4246,7 @@
         <v>157</v>
       </c>
       <c r="E130" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="131" spans="3:5">
@@ -4194,7 +4254,7 @@
         <v>158</v>
       </c>
       <c r="E131" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="132" spans="3:5">
@@ -4202,7 +4262,7 @@
         <v>159</v>
       </c>
       <c r="E132" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="133" spans="3:5">
@@ -4210,7 +4270,7 @@
         <v>160</v>
       </c>
       <c r="E133" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="134" spans="3:5">
@@ -4218,7 +4278,7 @@
         <v>161</v>
       </c>
       <c r="E134" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
     </row>
     <row r="135" spans="3:5">
@@ -4226,7 +4286,7 @@
         <v>162</v>
       </c>
       <c r="E135" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="136" spans="3:5">
@@ -4234,7 +4294,7 @@
         <v>163</v>
       </c>
       <c r="E136" t="s">
-        <v>88</v>
+        <v>529</v>
       </c>
     </row>
     <row r="137" spans="3:5">
@@ -4242,7 +4302,7 @@
         <v>164</v>
       </c>
       <c r="E137" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
     </row>
     <row r="138" spans="3:5">
@@ -4250,7 +4310,7 @@
         <v>165</v>
       </c>
       <c r="E138" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
     </row>
     <row r="139" spans="3:5">
@@ -4258,7 +4318,7 @@
         <v>166</v>
       </c>
       <c r="E139" t="s">
-        <v>362</v>
+        <v>91</v>
       </c>
     </row>
     <row r="140" spans="3:5">
@@ -4266,7 +4326,7 @@
         <v>167</v>
       </c>
       <c r="E140" t="s">
-        <v>367</v>
+        <v>532</v>
       </c>
     </row>
     <row r="141" spans="3:5">
@@ -4274,7 +4334,7 @@
         <v>168</v>
       </c>
       <c r="E141" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
     </row>
     <row r="142" spans="3:5">
@@ -4282,7 +4342,7 @@
         <v>169</v>
       </c>
       <c r="E142" t="s">
-        <v>529</v>
+        <v>365</v>
       </c>
     </row>
     <row r="143" spans="3:5">
@@ -4290,7 +4350,7 @@
         <v>170</v>
       </c>
       <c r="E143" t="s">
-        <v>530</v>
+        <v>370</v>
       </c>
     </row>
     <row r="144" spans="3:5">
@@ -4298,7 +4358,7 @@
         <v>171</v>
       </c>
       <c r="E144" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="145" spans="3:5">
@@ -4306,7 +4366,7 @@
         <v>172</v>
       </c>
       <c r="E145" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="146" spans="3:5">
@@ -4314,7 +4374,7 @@
         <v>173</v>
       </c>
       <c r="E146" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="147" spans="3:5">
@@ -4322,7 +4382,7 @@
         <v>174</v>
       </c>
       <c r="E147" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
     <row r="148" spans="3:5">
@@ -4330,7 +4390,7 @@
         <v>175</v>
       </c>
       <c r="E148" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="149" spans="3:5">
@@ -4338,7 +4398,7 @@
         <v>176</v>
       </c>
       <c r="E149" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="150" spans="3:5">
@@ -4346,7 +4406,7 @@
         <v>177</v>
       </c>
       <c r="E150" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="151" spans="3:5">
@@ -4354,7 +4414,7 @@
         <v>178</v>
       </c>
       <c r="E151" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="152" spans="3:5">
@@ -4362,7 +4422,7 @@
         <v>179</v>
       </c>
       <c r="E152" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="153" spans="3:5">
@@ -4370,23 +4430,32 @@
         <v>180</v>
       </c>
       <c r="E153" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
     </row>
     <row r="154" spans="3:5">
       <c r="C154" t="s">
         <v>181</v>
       </c>
+      <c r="E154" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="155" spans="3:5">
       <c r="C155" t="s">
         <v>182</v>
       </c>
+      <c r="E155" t="s">
+        <v>545</v>
+      </c>
     </row>
     <row r="156" spans="3:5">
       <c r="C156" t="s">
         <v>183</v>
       </c>
+      <c r="E156" t="s">
+        <v>546</v>
+      </c>
     </row>
     <row r="157" spans="3:5">
       <c r="C157" t="s">
@@ -5406,6 +5475,21 @@
     <row r="360" spans="3:3">
       <c r="C360" t="s">
         <v>387</v>
+      </c>
+    </row>
+    <row r="361" spans="3:3">
+      <c r="C361" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="362" spans="3:3">
+      <c r="C362" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="363" spans="3:3">
+      <c r="C363" t="s">
+        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -5420,37 +5504,37 @@
   <sheetData>
     <row r="1" spans="1:69">
       <c r="A1" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="B1" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="L1" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="O1" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="AA1" t="s">
-        <v>649</v>
+        <v>660</v>
       </c>
       <c r="AE1" t="s">
-        <v>654</v>
+        <v>665</v>
       </c>
       <c r="AI1" t="s">
-        <v>659</v>
+        <v>670</v>
       </c>
       <c r="AM1" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="AP1" t="s">
-        <v>668</v>
+        <v>679</v>
       </c>
       <c r="AS1" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="AZ1" t="s">
-        <v>680</v>
+        <v>691</v>
       </c>
       <c r="BM1" t="s">
         <v>16</v>
@@ -5458,211 +5542,211 @@
     </row>
     <row r="2" spans="1:69">
       <c r="A2" t="s">
-        <v>619</v>
+        <v>630</v>
       </c>
       <c r="B2" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="C2" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="D2" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="E2" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="F2" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
       <c r="G2" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="H2" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="I2" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="J2" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="K2" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="L2" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="M2" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="N2" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="O2" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
       <c r="P2" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
       <c r="Q2" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
       <c r="R2" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="S2" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="T2" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="U2" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="V2" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="W2" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="X2" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="Y2" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
       <c r="Z2" t="s">
-        <v>648</v>
+        <v>659</v>
       </c>
       <c r="AA2" t="s">
-        <v>650</v>
+        <v>661</v>
       </c>
       <c r="AB2" t="s">
-        <v>651</v>
+        <v>662</v>
       </c>
       <c r="AC2" t="s">
-        <v>652</v>
+        <v>663</v>
       </c>
       <c r="AD2" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="AE2" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
       <c r="AF2" t="s">
-        <v>656</v>
+        <v>667</v>
       </c>
       <c r="AG2" t="s">
-        <v>657</v>
+        <v>668</v>
       </c>
       <c r="AH2" t="s">
-        <v>658</v>
+        <v>669</v>
       </c>
       <c r="AI2" t="s">
-        <v>660</v>
+        <v>671</v>
       </c>
       <c r="AJ2" t="s">
-        <v>661</v>
+        <v>672</v>
       </c>
       <c r="AK2" t="s">
-        <v>662</v>
+        <v>673</v>
       </c>
       <c r="AL2" t="s">
-        <v>663</v>
+        <v>674</v>
       </c>
       <c r="AM2" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
       <c r="AN2" t="s">
-        <v>666</v>
+        <v>677</v>
       </c>
       <c r="AO2" t="s">
-        <v>667</v>
+        <v>678</v>
       </c>
       <c r="AP2" t="s">
-        <v>669</v>
+        <v>680</v>
       </c>
       <c r="AQ2" t="s">
-        <v>670</v>
+        <v>681</v>
       </c>
       <c r="AR2" t="s">
-        <v>671</v>
+        <v>682</v>
       </c>
       <c r="AS2" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
       <c r="AT2" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="AU2" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="AV2" t="s">
-        <v>676</v>
+        <v>687</v>
       </c>
       <c r="AW2" t="s">
-        <v>677</v>
+        <v>688</v>
       </c>
       <c r="AX2" t="s">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="AY2" t="s">
-        <v>679</v>
+        <v>690</v>
       </c>
       <c r="AZ2" t="s">
-        <v>681</v>
+        <v>692</v>
       </c>
       <c r="BA2" t="s">
-        <v>682</v>
+        <v>693</v>
       </c>
       <c r="BB2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
       <c r="BC2" t="s">
-        <v>684</v>
+        <v>695</v>
       </c>
       <c r="BD2" t="s">
-        <v>685</v>
+        <v>696</v>
       </c>
       <c r="BE2" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="BF2" t="s">
-        <v>687</v>
+        <v>698</v>
       </c>
       <c r="BG2" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="BH2" t="s">
-        <v>688</v>
+        <v>699</v>
       </c>
       <c r="BI2" t="s">
-        <v>689</v>
+        <v>700</v>
       </c>
       <c r="BJ2" t="s">
-        <v>690</v>
+        <v>701</v>
       </c>
       <c r="BK2" t="s">
-        <v>691</v>
+        <v>702</v>
       </c>
       <c r="BL2" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
       <c r="BM2" t="s">
-        <v>693</v>
+        <v>704</v>
       </c>
       <c r="BN2" t="s">
-        <v>694</v>
+        <v>705</v>
       </c>
       <c r="BO2" t="s">
-        <v>695</v>
+        <v>706</v>
       </c>
       <c r="BP2" t="s">
-        <v>696</v>
+        <v>707</v>
       </c>
       <c r="BQ2" t="s">
-        <v>697</v>
+        <v>708</v>
       </c>
     </row>
     <row r="3" spans="1:69">
@@ -6088,7 +6172,7 @@
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="G5" t="s">
         <v>24</v>
@@ -6502,228 +6586,228 @@
   <sheetData>
     <row r="1" spans="1:66">
       <c r="A1" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="B1" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="D1" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="J1" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
       <c r="AA1" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="AK1" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="AV1" t="s">
-        <v>680</v>
+        <v>691</v>
       </c>
       <c r="BM1" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
     </row>
     <row r="2" spans="1:66">
       <c r="A2" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
       <c r="B2" t="s">
-        <v>699</v>
+        <v>710</v>
       </c>
       <c r="C2" t="s">
-        <v>700</v>
+        <v>711</v>
       </c>
       <c r="D2" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="E2" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="F2" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="G2" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
       <c r="H2" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="I2" t="s">
-        <v>707</v>
+        <v>718</v>
       </c>
       <c r="J2" t="s">
-        <v>709</v>
+        <v>720</v>
       </c>
       <c r="K2" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
       <c r="L2" t="s">
-        <v>711</v>
+        <v>722</v>
       </c>
       <c r="M2" t="s">
-        <v>712</v>
+        <v>723</v>
       </c>
       <c r="N2" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
       <c r="O2" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
       <c r="P2" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
       <c r="Q2" t="s">
-        <v>716</v>
+        <v>727</v>
       </c>
       <c r="R2" t="s">
-        <v>717</v>
+        <v>728</v>
       </c>
       <c r="S2" t="s">
-        <v>718</v>
+        <v>729</v>
       </c>
       <c r="T2" t="s">
-        <v>719</v>
+        <v>730</v>
       </c>
       <c r="U2" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="V2" t="s">
-        <v>721</v>
+        <v>732</v>
       </c>
       <c r="W2" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="X2" t="s">
-        <v>723</v>
+        <v>734</v>
       </c>
       <c r="Y2" t="s">
-        <v>724</v>
+        <v>735</v>
       </c>
       <c r="Z2" t="s">
-        <v>725</v>
+        <v>736</v>
       </c>
       <c r="AA2" t="s">
-        <v>727</v>
+        <v>738</v>
       </c>
       <c r="AB2" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="AC2" t="s">
-        <v>729</v>
+        <v>740</v>
       </c>
       <c r="AD2" t="s">
-        <v>730</v>
+        <v>741</v>
       </c>
       <c r="AE2" t="s">
-        <v>731</v>
+        <v>742</v>
       </c>
       <c r="AF2" t="s">
-        <v>732</v>
+        <v>743</v>
       </c>
       <c r="AG2" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="AH2" t="s">
-        <v>734</v>
+        <v>745</v>
       </c>
       <c r="AI2" t="s">
-        <v>735</v>
+        <v>746</v>
       </c>
       <c r="AJ2" t="s">
-        <v>736</v>
+        <v>747</v>
       </c>
       <c r="AK2" t="s">
-        <v>737</v>
+        <v>748</v>
       </c>
       <c r="AL2" t="s">
-        <v>738</v>
+        <v>749</v>
       </c>
       <c r="AM2" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="AN2" t="s">
-        <v>740</v>
+        <v>751</v>
       </c>
       <c r="AO2" t="s">
-        <v>741</v>
+        <v>752</v>
       </c>
       <c r="AP2" t="s">
-        <v>742</v>
+        <v>753</v>
       </c>
       <c r="AQ2" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="AR2" t="s">
-        <v>744</v>
+        <v>755</v>
       </c>
       <c r="AS2" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
       <c r="AT2" t="s">
-        <v>746</v>
+        <v>757</v>
       </c>
       <c r="AU2" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="AV2" t="s">
-        <v>748</v>
+        <v>759</v>
       </c>
       <c r="AW2" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="AX2" t="s">
-        <v>750</v>
+        <v>761</v>
       </c>
       <c r="AY2" t="s">
-        <v>751</v>
+        <v>762</v>
       </c>
       <c r="AZ2" t="s">
-        <v>752</v>
+        <v>763</v>
       </c>
       <c r="BA2" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="BB2" t="s">
-        <v>754</v>
+        <v>765</v>
       </c>
       <c r="BC2" t="s">
-        <v>755</v>
+        <v>766</v>
       </c>
       <c r="BD2" t="s">
-        <v>756</v>
+        <v>767</v>
       </c>
       <c r="BE2" t="s">
-        <v>757</v>
+        <v>768</v>
       </c>
       <c r="BF2" t="s">
-        <v>758</v>
+        <v>769</v>
       </c>
       <c r="BG2" t="s">
-        <v>759</v>
+        <v>770</v>
       </c>
       <c r="BH2" t="s">
-        <v>760</v>
+        <v>771</v>
       </c>
       <c r="BI2" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="BJ2" t="s">
-        <v>762</v>
+        <v>773</v>
       </c>
       <c r="BK2" t="s">
-        <v>763</v>
+        <v>774</v>
       </c>
       <c r="BL2" t="s">
-        <v>764</v>
+        <v>775</v>
       </c>
       <c r="BM2" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="BN2" t="s">
-        <v>767</v>
+        <v>778</v>
       </c>
     </row>
     <row r="3" spans="1:66">
@@ -7197,7 +7281,7 @@
         <v>20</v>
       </c>
       <c r="Z5" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="AA5" t="s">
         <v>18</v>

</xml_diff>